<commit_message>
feat: harden modeling paper production and rebuild 2025A
</commit_message>
<xml_diff>
--- a/projects/2025-a-smoke-screen/outputs/result1.xlsx
+++ b/projects/2025-a-smoke-screen/outputs/result1.xlsx
@@ -528,98 +528,98 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>179.8520077475987</v>
+        <v>179.5761916428091</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>128.0681045900068</v>
+        <v>124.3019426375411</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>17799.30433113121</v>
+        <v>17798.31072422191</v>
       </c>
       <c r="E2" t="n">
-        <v>0.001796883342007471</v>
+        <v>0.01249554950991511</v>
       </c>
       <c r="F2" t="n">
         <v>1800</v>
       </c>
       <c r="G2" t="n">
-        <v>17797.70433159744</v>
+        <v>17797.41416630796</v>
       </c>
       <c r="H2" t="n">
-        <v>0.005929614643422495</v>
+        <v>0.01912737596928853</v>
       </c>
       <c r="I2" t="n">
-        <v>1799.999235184421</v>
+        <v>1799.99974507014</v>
       </c>
       <c r="J2" t="n">
-        <v>2.60639569132208</v>
+        <v>2.604257461644922</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>179.8520077475987</v>
+        <v>179.5761916428091</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>128.0681045900068</v>
+        <v>124.3019426375411</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>17534.82895428152</v>
+        <v>17566.29815200786</v>
       </c>
       <c r="E3" t="n">
-        <v>0.684925625125224</v>
+        <v>1.728689329488997</v>
       </c>
       <c r="F3" t="n">
         <v>1800</v>
       </c>
       <c r="G3" t="n">
-        <v>16962.29066004981</v>
+        <v>17066.67279708547</v>
       </c>
       <c r="H3" t="n">
-        <v>2.163767887191465</v>
+        <v>5.424411152901882</v>
       </c>
       <c r="I3" t="n">
-        <v>1702.067668716495</v>
+        <v>1720.831402830285</v>
       </c>
       <c r="J3" t="n">
-        <v>3.351768379791793</v>
+        <v>2.508251600646662</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>179.8520077475987</v>
+        <v>179.5761916428091</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>128.0681045900068</v>
+        <v>124.3019426375411</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>17328.31138447371</v>
+        <v>17242.35739126497</v>
       </c>
       <c r="E4" t="n">
-        <v>1.21835179620926</v>
+        <v>4.124874645497287</v>
       </c>
       <c r="F4" t="n">
         <v>1800</v>
       </c>
       <c r="G4" t="n">
-        <v>16658.04140394654</v>
+        <v>16589.67195815951</v>
       </c>
       <c r="H4" t="n">
-        <v>2.949630881266809</v>
+        <v>8.952779745161948</v>
       </c>
       <c r="I4" t="n">
-        <v>1665.780211069678</v>
+        <v>1664.894866776935</v>
       </c>
       <c r="J4" t="n">
-        <v>2.302923888173989</v>
+        <v>1.701515093753384</v>
       </c>
     </row>
     <row r="5">

</xml_diff>